<commit_message>
Refactor in line with updated project schema
</commit_message>
<xml_diff>
--- a/tabular/legacy-list.xlsx
+++ b/tabular/legacy-list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rob/Projects/erv/ERVdb-HomoSapiens/tabular/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78FF3E04-AFE8-F84C-A0D0-FAAEBD36B583}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE81D4B9-E08D-2840-A2AB-18C582FF9BD2}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1280" yWindow="1000" windowWidth="27140" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1360" uniqueCount="500">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1370" uniqueCount="502">
   <si>
     <t>organism</t>
   </si>
@@ -1521,6 +1521,12 @@
   </si>
   <si>
     <t>HERV-K 113</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>found?</t>
   </si>
 </sst>
 </file>
@@ -2376,15 +2382,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O143"/>
+  <dimension ref="A1:P152"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="47.1640625" customWidth="1"/>
     <col min="5" max="5" width="34" customWidth="1"/>
     <col min="6" max="6" width="51.6640625" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" customWidth="1"/>
+    <col min="8" max="8" width="18.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2430,8 +2438,11 @@
       <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P1" s="2" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -2463,7 +2474,7 @@
         <v>13467826</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -2504,7 +2515,7 @@
         <v>46856998</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -2548,7 +2559,7 @@
         <v>75849143</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -2589,7 +2600,7 @@
         <v>89397564</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -2627,7 +2638,7 @@
         <v>110252173</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>15</v>
       </c>
@@ -2665,7 +2676,7 @@
         <v>150631285</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -2709,7 +2720,7 @@
         <v>155605636</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -2753,7 +2764,7 @@
         <v>160669806</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>15</v>
       </c>
@@ -2785,7 +2796,7 @@
         <v>166580258</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -2826,7 +2837,7 @@
         <v>178112194</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>15</v>
       </c>
@@ -2867,7 +2878,7 @@
         <v>205844935</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>15</v>
       </c>
@@ -2908,7 +2919,7 @@
         <v>227821260</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>15</v>
       </c>
@@ -2952,7 +2963,7 @@
         <v>6875603</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>15</v>
       </c>
@@ -2987,7 +2998,7 @@
         <v>27183380</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>15</v>
       </c>
@@ -7506,7 +7517,7 @@
         <v>8055725</v>
       </c>
     </row>
-    <row r="129" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>15</v>
       </c>
@@ -7547,7 +7558,7 @@
         <v>12081622</v>
       </c>
     </row>
-    <row r="130" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
         <v>15</v>
       </c>
@@ -7588,7 +7599,7 @@
         <v>12350376</v>
       </c>
     </row>
-    <row r="131" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
         <v>15</v>
       </c>
@@ -7620,7 +7631,7 @@
         <v>47183661</v>
       </c>
     </row>
-    <row r="132" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
         <v>15</v>
       </c>
@@ -7658,7 +7669,7 @@
         <v>54988656</v>
       </c>
     </row>
-    <row r="133" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
         <v>15</v>
       </c>
@@ -7699,7 +7710,7 @@
         <v>81655427</v>
       </c>
     </row>
-    <row r="134" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
         <v>15</v>
       </c>
@@ -7731,7 +7742,7 @@
         <v>146254211</v>
       </c>
     </row>
-    <row r="135" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
         <v>15</v>
       </c>
@@ -7772,7 +7783,7 @@
         <v>21932738</v>
       </c>
     </row>
-    <row r="136" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
         <v>15</v>
       </c>
@@ -7813,7 +7824,7 @@
         <v>35642824</v>
       </c>
     </row>
-    <row r="137" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
         <v>15</v>
       </c>
@@ -7854,7 +7865,7 @@
         <v>90659200</v>
       </c>
     </row>
-    <row r="138" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
         <v>15</v>
       </c>
@@ -7886,7 +7897,7 @@
         <v>131619736</v>
       </c>
     </row>
-    <row r="139" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
         <v>15</v>
       </c>
@@ -7918,7 +7929,7 @@
         <v>139684228</v>
       </c>
     </row>
-    <row r="140" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
         <v>15</v>
       </c>
@@ -7962,7 +7973,7 @@
         <v>4463549</v>
       </c>
     </row>
-    <row r="141" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
         <v>15</v>
       </c>
@@ -8006,7 +8017,7 @@
         <v>106298101</v>
       </c>
     </row>
-    <row r="142" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
         <v>15</v>
       </c>
@@ -8038,7 +8049,7 @@
         <v>153819562</v>
       </c>
     </row>
-    <row r="143" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
         <v>15</v>
       </c>
@@ -8077,6 +8088,395 @@
       </c>
       <c r="N143">
         <v>23206610</v>
+      </c>
+    </row>
+    <row r="144" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A144" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B144" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C144" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D144" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="E144" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="F144" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="G144" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="H144" s="3"/>
+      <c r="I144" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="J144" s="3">
+        <v>3272</v>
+      </c>
+      <c r="K144" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="L144" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="M144" s="3">
+        <v>229406344</v>
+      </c>
+      <c r="N144" s="3">
+        <v>229408495</v>
+      </c>
+      <c r="P144" s="3" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="145" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A145" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B145" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C145" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D145" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="E145" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="F145" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="G145" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="H145" s="3">
+        <v>4</v>
+      </c>
+      <c r="I145" s="3"/>
+      <c r="J145" s="3"/>
+      <c r="K145" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L145" s="3" t="s">
+        <v>365</v>
+      </c>
+      <c r="M145" s="3">
+        <v>89372203</v>
+      </c>
+      <c r="N145" s="3">
+        <v>89375974</v>
+      </c>
+      <c r="P145" s="3" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="146" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A146" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B146" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C146" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D146" s="3" t="s">
+        <v>456</v>
+      </c>
+      <c r="E146" s="3"/>
+      <c r="F146" s="3" t="s">
+        <v>457</v>
+      </c>
+      <c r="G146" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H146" s="3"/>
+      <c r="I146" s="3"/>
+      <c r="J146" s="3"/>
+      <c r="K146" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L146" s="3" t="s">
+        <v>452</v>
+      </c>
+      <c r="M146" s="3">
+        <v>12316492</v>
+      </c>
+      <c r="N146" s="3">
+        <v>12326007</v>
+      </c>
+      <c r="P146" s="3" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="147" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A147" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B147" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C147" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D147" s="3" t="s">
+        <v>465</v>
+      </c>
+      <c r="E147" s="3" t="s">
+        <v>466</v>
+      </c>
+      <c r="F147" s="3"/>
+      <c r="G147" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="H147" s="3">
+        <v>20</v>
+      </c>
+      <c r="I147" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="J147" s="3">
+        <v>106144604</v>
+      </c>
+      <c r="K147" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L147" s="3" t="s">
+        <v>452</v>
+      </c>
+      <c r="M147" s="3">
+        <v>74734099</v>
+      </c>
+      <c r="N147" s="3">
+        <v>74734838</v>
+      </c>
+      <c r="P147" s="3" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="148" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A148" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B148" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C148" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D148" s="3" t="s">
+        <v>375</v>
+      </c>
+      <c r="E148" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="F148" s="3" t="s">
+        <v>377</v>
+      </c>
+      <c r="G148" s="3"/>
+      <c r="H148" s="3">
+        <v>1610</v>
+      </c>
+      <c r="I148" s="3" t="s">
+        <v>378</v>
+      </c>
+      <c r="J148" s="3">
+        <v>101928353</v>
+      </c>
+      <c r="K148" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L148" s="3" t="s">
+        <v>365</v>
+      </c>
+      <c r="M148" s="3">
+        <v>71103905</v>
+      </c>
+      <c r="N148" s="3">
+        <v>71109120</v>
+      </c>
+      <c r="P148" s="3" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="149" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A149" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B149" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C149" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D149" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="E149" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="F149" s="3"/>
+      <c r="G149" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H149" s="3">
+        <v>30</v>
+      </c>
+      <c r="I149" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="J149" s="3">
+        <v>106144591</v>
+      </c>
+      <c r="K149" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L149" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="M149" s="3">
+        <v>187385634</v>
+      </c>
+      <c r="N149" s="3">
+        <v>187387099</v>
+      </c>
+      <c r="P149" s="3" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="150" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A150" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B150" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C150" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D150" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E150" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F150" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="G150" s="3"/>
+      <c r="H150" s="3">
+        <v>1</v>
+      </c>
+      <c r="I150" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="J150" s="3">
+        <v>339476</v>
+      </c>
+      <c r="K150" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L150" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="M150" s="3">
+        <v>187610358</v>
+      </c>
+      <c r="N150" s="3">
+        <v>187612992</v>
+      </c>
+      <c r="P150" s="3" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="151" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A151" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B151" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C151" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D151" s="3" t="s">
+        <v>482</v>
+      </c>
+      <c r="E151" s="3"/>
+      <c r="F151" s="3" t="s">
+        <v>498</v>
+      </c>
+      <c r="G151" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H151" s="3">
+        <v>105</v>
+      </c>
+      <c r="I151" s="3"/>
+      <c r="J151" s="3"/>
+      <c r="K151" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L151" s="3" t="s">
+        <v>483</v>
+      </c>
+      <c r="M151" s="3">
+        <v>175210</v>
+      </c>
+      <c r="N151" s="3">
+        <v>176178</v>
+      </c>
+      <c r="P151" s="3" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="152" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A152" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B152" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C152" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D152" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="E152" s="3"/>
+      <c r="F152" s="3" t="s">
+        <v>499</v>
+      </c>
+      <c r="G152" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H152" s="3">
+        <v>113</v>
+      </c>
+      <c r="I152" s="3"/>
+      <c r="J152" s="3"/>
+      <c r="K152" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="L152" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="M152" s="3">
+        <v>21841536</v>
+      </c>
+      <c r="N152" s="3">
+        <v>21841542</v>
+      </c>
+      <c r="P152" s="3" t="s">
+        <v>500</v>
       </c>
     </row>
   </sheetData>
@@ -8086,7 +8486,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCBE97ED-1BA3-824F-A08D-55E4843F8392}">
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="45.6640625" customWidth="1"/>
@@ -8140,377 +8540,6 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="J2" s="3">
-        <v>3272</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="M2" s="3">
-        <v>229406344</v>
-      </c>
-      <c r="N2" s="3">
-        <v>229408495</v>
-      </c>
-      <c r="O2" s="3"/>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>390</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>391</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>393</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>175</v>
-      </c>
-      <c r="H3" s="3">
-        <v>4</v>
-      </c>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>365</v>
-      </c>
-      <c r="M3" s="3">
-        <v>89372203</v>
-      </c>
-      <c r="N3" s="3">
-        <v>89375974</v>
-      </c>
-      <c r="O3" s="3"/>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>456</v>
-      </c>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3" t="s">
-        <v>457</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>452</v>
-      </c>
-      <c r="M4" s="3">
-        <v>12316492</v>
-      </c>
-      <c r="N4" s="3">
-        <v>12326007</v>
-      </c>
-      <c r="O4" s="3"/>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>465</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>466</v>
-      </c>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="H5" s="3">
-        <v>20</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>467</v>
-      </c>
-      <c r="J5" s="3">
-        <v>106144604</v>
-      </c>
-      <c r="K5" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>452</v>
-      </c>
-      <c r="M5" s="3">
-        <v>74734099</v>
-      </c>
-      <c r="N5" s="3">
-        <v>74734838</v>
-      </c>
-      <c r="O5" s="3"/>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>375</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>376</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>377</v>
-      </c>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3">
-        <v>1610</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>378</v>
-      </c>
-      <c r="J6" s="3">
-        <v>101928353</v>
-      </c>
-      <c r="K6" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="L6" s="3" t="s">
-        <v>365</v>
-      </c>
-      <c r="M6" s="3">
-        <v>71103905</v>
-      </c>
-      <c r="N6" s="3">
-        <v>71109120</v>
-      </c>
-      <c r="O6" s="3"/>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>259</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>260</v>
-      </c>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H7" s="3">
-        <v>30</v>
-      </c>
-      <c r="I7" s="3" t="s">
-        <v>261</v>
-      </c>
-      <c r="J7" s="3">
-        <v>106144591</v>
-      </c>
-      <c r="K7" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="L7" s="3" t="s">
-        <v>241</v>
-      </c>
-      <c r="M7" s="3">
-        <v>187385634</v>
-      </c>
-      <c r="N7" s="3">
-        <v>187387099</v>
-      </c>
-      <c r="O7" s="3"/>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A8" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3">
-        <v>1</v>
-      </c>
-      <c r="I8" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="J8" s="3">
-        <v>339476</v>
-      </c>
-      <c r="K8" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="L8" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="M8" s="3">
-        <v>187610358</v>
-      </c>
-      <c r="N8" s="3">
-        <v>187612992</v>
-      </c>
-      <c r="O8" s="3"/>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A9" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>482</v>
-      </c>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3" t="s">
-        <v>498</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H9" s="3">
-        <v>105</v>
-      </c>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="L9" s="3" t="s">
-        <v>483</v>
-      </c>
-      <c r="M9" s="3">
-        <v>175210</v>
-      </c>
-      <c r="N9" s="3">
-        <v>176178</v>
-      </c>
-      <c r="O9" s="3"/>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A10" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3" t="s">
-        <v>499</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H10" s="3">
-        <v>113</v>
-      </c>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="L10" s="3" t="s">
-        <v>191</v>
-      </c>
-      <c r="M10" s="3">
-        <v>21841536</v>
-      </c>
-      <c r="N10" s="3">
-        <v>21841542</v>
-      </c>
-      <c r="O10" s="3"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>